<commit_message>
streamlit to tkinter changes
</commit_message>
<xml_diff>
--- a/models/hv/data/scan_log.xlsx
+++ b/models/hv/data/scan_log.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3036" yWindow="2340" windowWidth="11268" windowHeight="9900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HV Dummy" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="HV Dummy" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2059,6 +2059,76 @@
       <c r="Q22" s="18" t="inlineStr"/>
       <c r="R22" s="18" t="inlineStr"/>
     </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>10:40:01 PM</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>00200</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>ABA51202609241A00200</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260076</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260077</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260078</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>VX156610-E1611109G260079</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>INTEGRATION OK</t>
+        </is>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202609241A00200</t>
+        </is>
+      </c>
+      <c r="N23" s="10" t="inlineStr"/>
+      <c r="O23" s="10" t="inlineStr"/>
+      <c r="P23" s="10" t="inlineStr"/>
+      <c r="Q23" s="10" t="inlineStr"/>
+      <c r="R23" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>